<commit_message>
Refactor quote generation workflow and layout handling
</commit_message>
<xml_diff>
--- a/docs/Quotation-Cost-Template-V1.1.xlsx
+++ b/docs/Quotation-Cost-Template-V1.1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aaa/Konceptliving Dropbox/Konceptliving Team Folder/KONCEPT QUOTATION/Template/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\xPass\GitHub Projects\koncept-quote-auto-generator\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB79C0DD-FACC-494E-8BC4-640909092A90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49393CF8-8C7E-48F1-AF17-D06C518ACAEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="25600" windowHeight="14040" xr2:uid="{C830D79F-9B19-7342-9B39-F4DE5434FDDB}"/>
+    <workbookView xWindow="-109" yWindow="-109" windowWidth="26301" windowHeight="14169" xr2:uid="{C830D79F-9B19-7342-9B39-F4DE5434FDDB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -19,17 +19,6 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -395,15 +384,9 @@
     <t>HQI Floodlight</t>
   </si>
   <si>
-    <t>nos. LED recess dowlight 3"</t>
-  </si>
-  <si>
     <t>Downlight</t>
   </si>
   <si>
-    <t>nos. LED recess dowlight 6"</t>
-  </si>
-  <si>
     <t>nos.13Amp/230V SP 50Hz AC Socket (Max 800W) (Not for lighting use) </t>
   </si>
   <si>
@@ -702,6 +685,12 @@
   </si>
   <si>
     <t>COFFEE PER DAY</t>
+  </si>
+  <si>
+    <t>nos. LED recess downlight 3"</t>
+  </si>
+  <si>
+    <t>nos. LED recess downlight 6"</t>
   </si>
 </sst>
 </file>
@@ -2691,18 +2680,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2355A233-406B-9740-B1B1-24942A627A7E}">
   <dimension ref="A2:O278"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.77734375" defaultRowHeight="15.65" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="10.83203125" style="2"/>
+    <col min="1" max="2" width="10.77734375" style="2"/>
     <col min="3" max="3" width="44.33203125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="18.77734375" style="2" customWidth="1"/>
     <col min="5" max="5" width="13" style="2" customWidth="1"/>
-    <col min="6" max="11" width="10.83203125" style="2"/>
+    <col min="6" max="11" width="10.77734375" style="2"/>
     <col min="12" max="12" width="25.33203125" style="10" customWidth="1"/>
-    <col min="13" max="16384" width="10.83203125" style="2"/>
+    <col min="13" max="16384" width="10.77734375" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="5">
         <v>1</v>
       </c>
@@ -2727,7 +2716,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="18" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12" ht="18.350000000000001" x14ac:dyDescent="0.25">
       <c r="C4" s="8" t="s">
         <v>6</v>
       </c>
@@ -2749,7 +2738,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="18" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:12" ht="18.350000000000001" x14ac:dyDescent="0.25">
       <c r="C6" s="8" t="s">
         <v>8</v>
       </c>
@@ -2771,7 +2760,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="18" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:12" ht="18.350000000000001" x14ac:dyDescent="0.25">
       <c r="C8" s="8" t="s">
         <v>10</v>
       </c>
@@ -2793,7 +2782,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="18" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:12" ht="18.350000000000001" x14ac:dyDescent="0.25">
       <c r="C10" s="8" t="s">
         <v>12</v>
       </c>
@@ -2815,7 +2804,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="18" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:12" ht="18.350000000000001" x14ac:dyDescent="0.25">
       <c r="C12" s="8" t="s">
         <v>14</v>
       </c>
@@ -2837,7 +2826,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="18" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:12" ht="18.350000000000001" x14ac:dyDescent="0.25">
       <c r="C14" s="8" t="s">
         <v>16</v>
       </c>
@@ -2859,7 +2848,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>2</v>
       </c>
@@ -2868,9 +2857,9 @@
       </c>
       <c r="D17" s="3"/>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C19" s="2" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="F19" s="2">
         <f>B19*H19*J19</f>
@@ -2886,7 +2875,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C20" s="2" t="s">
         <v>20</v>
       </c>
@@ -2894,9 +2883,9 @@
         <v>21</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C22" s="2" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="F22" s="2">
         <f>B22*H22*J22</f>
@@ -2912,7 +2901,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C23" s="2" t="s">
         <v>31</v>
       </c>
@@ -2920,9 +2909,9 @@
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C25" s="2" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F25" s="2">
         <f>B25*H25*J25</f>
@@ -2938,7 +2927,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C26" s="2" t="s">
         <v>25</v>
       </c>
@@ -2946,9 +2935,9 @@
         <v>21</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C28" s="2" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F28" s="2">
         <f>B28*H28*J28</f>
@@ -2964,7 +2953,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C29" s="2" t="s">
         <v>22</v>
       </c>
@@ -2972,7 +2961,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C31" s="2" t="s">
         <v>27</v>
       </c>
@@ -2990,7 +2979,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C32" s="2" t="s">
         <v>20</v>
       </c>
@@ -2998,7 +2987,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="34" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="34" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C34" s="2" t="s">
         <v>27</v>
       </c>
@@ -3016,7 +3005,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="35" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="35" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C35" s="2" t="s">
         <v>22</v>
       </c>
@@ -3024,7 +3013,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="37" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="37" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C37" s="2" t="s">
         <v>28</v>
       </c>
@@ -3042,7 +3031,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="38" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="38" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C38" s="2" t="s">
         <v>20</v>
       </c>
@@ -3050,7 +3039,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="40" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="40" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C40" s="2" t="s">
         <v>28</v>
       </c>
@@ -3068,7 +3057,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="41" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="41" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C41" s="2" t="s">
         <v>22</v>
       </c>
@@ -3076,7 +3065,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="44" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="44" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C44" s="2" t="s">
         <v>29</v>
       </c>
@@ -3094,7 +3083,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="45" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="45" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C45" s="2" t="s">
         <v>20</v>
       </c>
@@ -3102,7 +3091,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="47" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="47" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C47" s="2" t="s">
         <v>29</v>
       </c>
@@ -3120,7 +3109,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="48" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="48" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C48" s="2" t="s">
         <v>31</v>
       </c>
@@ -3128,7 +3117,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="50" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="50" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C50" s="2" t="s">
         <v>32</v>
       </c>
@@ -3146,7 +3135,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="51" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="51" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C51" s="2" t="s">
         <v>20</v>
       </c>
@@ -3154,7 +3143,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="53" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="53" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C53" s="2" t="s">
         <v>32</v>
       </c>
@@ -3172,7 +3161,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="54" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="54" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C54" s="2" t="s">
         <v>31</v>
       </c>
@@ -3180,7 +3169,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="56" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="56" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C56" s="2" t="s">
         <v>34</v>
       </c>
@@ -3198,12 +3187,12 @@
         <v>35</v>
       </c>
     </row>
-    <row r="57" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="57" spans="3:12" x14ac:dyDescent="0.25">
       <c r="L57" s="10" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="59" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="59" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C59" s="2" t="s">
         <v>36</v>
       </c>
@@ -3221,14 +3210,14 @@
         <v>35</v>
       </c>
     </row>
-    <row r="60" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="60" spans="3:12" x14ac:dyDescent="0.25">
       <c r="L60" s="10" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="62" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="62" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C62" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="F62" s="2">
         <f>B62*H62*J62</f>
@@ -3242,15 +3231,15 @@
         <v>1.5</v>
       </c>
       <c r="L62" s="10" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="63" spans="3:12" x14ac:dyDescent="0.2">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="63" spans="3:12" x14ac:dyDescent="0.25">
       <c r="L63" s="10" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="65" spans="3:12" x14ac:dyDescent="0.2">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="65" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C65" s="2" t="s">
         <v>37</v>
       </c>
@@ -3268,12 +3257,12 @@
         <v>38</v>
       </c>
     </row>
-    <row r="66" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="66" spans="3:12" x14ac:dyDescent="0.25">
       <c r="L66" s="10" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="68" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="68" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C68" s="2" t="s">
         <v>39</v>
       </c>
@@ -3291,12 +3280,12 @@
         <v>38</v>
       </c>
     </row>
-    <row r="69" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="69" spans="3:12" x14ac:dyDescent="0.25">
       <c r="L69" s="10" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="71" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="71" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C71" s="2" t="s">
         <v>40</v>
       </c>
@@ -3314,12 +3303,12 @@
         <v>41</v>
       </c>
     </row>
-    <row r="72" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="72" spans="3:12" x14ac:dyDescent="0.25">
       <c r="L72" s="10" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="74" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="74" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C74" s="2" t="s">
         <v>42</v>
       </c>
@@ -3337,12 +3326,12 @@
         <v>41</v>
       </c>
     </row>
-    <row r="75" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="75" spans="3:12" x14ac:dyDescent="0.25">
       <c r="L75" s="10" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="77" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="77" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C77" s="2" t="s">
         <v>43</v>
       </c>
@@ -3360,7 +3349,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="81" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A81" s="1">
         <v>3</v>
       </c>
@@ -3369,12 +3358,12 @@
       </c>
       <c r="D81" s="3"/>
     </row>
-    <row r="82" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A82" s="1"/>
       <c r="C82" s="3"/>
       <c r="D82" s="3"/>
     </row>
-    <row r="83" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A83" s="1"/>
       <c r="C83" s="2" t="s">
         <v>46</v>
@@ -3393,7 +3382,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="84" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A84" s="1"/>
       <c r="C84" s="2" t="s">
         <v>48</v>
@@ -3402,10 +3391,10 @@
         <v>21</v>
       </c>
     </row>
-    <row r="85" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A85" s="1"/>
     </row>
-    <row r="86" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A86" s="1"/>
       <c r="C86" s="2" t="s">
         <v>46</v>
@@ -3424,7 +3413,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="87" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A87" s="1"/>
       <c r="C87" s="2" t="s">
         <v>31</v>
@@ -3433,10 +3422,10 @@
         <v>49</v>
       </c>
     </row>
-    <row r="88" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A88" s="1"/>
     </row>
-    <row r="89" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A89" s="1"/>
       <c r="C89" s="2" t="s">
         <v>50</v>
@@ -3455,7 +3444,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="90" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A90" s="1"/>
       <c r="C90" s="2" t="s">
         <v>48</v>
@@ -3464,10 +3453,10 @@
         <v>21</v>
       </c>
     </row>
-    <row r="91" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A91" s="1"/>
     </row>
-    <row r="92" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A92" s="1"/>
       <c r="C92" s="2" t="s">
         <v>50</v>
@@ -3486,7 +3475,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="93" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A93" s="1"/>
       <c r="C93" s="2" t="s">
         <v>31</v>
@@ -3495,10 +3484,10 @@
         <v>49</v>
       </c>
     </row>
-    <row r="94" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A94" s="1"/>
     </row>
-    <row r="95" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A95" s="1"/>
       <c r="C95" s="2" t="s">
         <v>52</v>
@@ -3517,7 +3506,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="96" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A96" s="1"/>
       <c r="C96" s="2" t="s">
         <v>48</v>
@@ -3526,10 +3515,10 @@
         <v>21</v>
       </c>
     </row>
-    <row r="97" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A97" s="1"/>
     </row>
-    <row r="98" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A98" s="1"/>
       <c r="C98" s="2" t="s">
         <v>52</v>
@@ -3548,7 +3537,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="99" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A99" s="1"/>
       <c r="C99" s="2" t="s">
         <v>31</v>
@@ -3557,10 +3546,10 @@
         <v>49</v>
       </c>
     </row>
-    <row r="100" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A100" s="1"/>
     </row>
-    <row r="101" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A101" s="1"/>
       <c r="C101" s="2" t="s">
         <v>54</v>
@@ -3582,10 +3571,10 @@
         <v>55</v>
       </c>
     </row>
-    <row r="102" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A102" s="1"/>
     </row>
-    <row r="104" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A104" s="1">
         <v>4</v>
       </c>
@@ -3594,7 +3583,7 @@
       </c>
       <c r="D104" s="3"/>
     </row>
-    <row r="106" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C106" s="2" t="s">
         <v>57</v>
       </c>
@@ -3615,7 +3604,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="108" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C108" s="2" t="s">
         <v>59</v>
       </c>
@@ -3636,16 +3625,16 @@
         <v>60</v>
       </c>
     </row>
-    <row r="109" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C109" s="2" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="110" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C110" s="4"/>
       <c r="D110" s="4"/>
     </row>
-    <row r="111" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C111" s="2" t="s">
         <v>62</v>
       </c>
@@ -3666,7 +3655,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="113" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B113" s="2">
         <v>1</v>
       </c>
@@ -3690,7 +3679,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="115" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C115" s="2" t="s">
         <v>66</v>
       </c>
@@ -3711,7 +3700,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="116" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C116" s="2" t="s">
         <v>20</v>
       </c>
@@ -3719,7 +3708,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="118" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C118" s="2" t="s">
         <v>66</v>
       </c>
@@ -3740,7 +3729,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="119" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C119" s="2" t="s">
         <v>31</v>
       </c>
@@ -3748,7 +3737,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="121" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C121" s="2" t="s">
         <v>66</v>
       </c>
@@ -3769,17 +3758,17 @@
         <v>68</v>
       </c>
     </row>
-    <row r="122" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C122" s="2" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="123" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C123" s="2" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="125" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C125" s="2" t="s">
         <v>71</v>
       </c>
@@ -3808,7 +3797,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="126" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:15" x14ac:dyDescent="0.25">
       <c r="N126" s="2">
         <v>1000</v>
       </c>
@@ -3817,7 +3806,7 @@
         <v>14.705882352941176</v>
       </c>
     </row>
-    <row r="128" spans="1:15" ht="17" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:15" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A128" s="1">
         <v>5</v>
       </c>
@@ -3826,7 +3815,7 @@
       </c>
       <c r="D128" s="3"/>
     </row>
-    <row r="130" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="130" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C130" s="2" t="s">
         <v>73</v>
       </c>
@@ -3847,7 +3836,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="132" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="132" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C132" s="2" t="s">
         <v>75</v>
       </c>
@@ -3868,7 +3857,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="134" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="134" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C134" s="2" t="s">
         <v>77</v>
       </c>
@@ -3889,7 +3878,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="136" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="136" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C136" s="2" t="s">
         <v>79</v>
       </c>
@@ -3910,9 +3899,9 @@
         <v>80</v>
       </c>
     </row>
-    <row r="138" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="138" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C138" s="2" t="s">
-        <v>81</v>
+        <v>182</v>
       </c>
       <c r="F138" s="2">
         <f t="shared" ref="F138" si="12">B138*H138*I138*J138</f>
@@ -3928,12 +3917,12 @@
         <v>1.5</v>
       </c>
       <c r="L138" s="10" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="140" spans="3:12" x14ac:dyDescent="0.2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="140" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C140" s="2" t="s">
-        <v>83</v>
+        <v>183</v>
       </c>
       <c r="F140" s="2">
         <f t="shared" ref="F140" si="13">B140*H140*I140*J140</f>
@@ -3949,12 +3938,12 @@
         <v>1.5</v>
       </c>
       <c r="L140" s="10" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="142" spans="3:12" x14ac:dyDescent="0.25">
+      <c r="C142" s="2" t="s">
         <v>82</v>
-      </c>
-    </row>
-    <row r="142" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="C142" s="2" t="s">
-        <v>84</v>
       </c>
       <c r="F142" s="2">
         <f t="shared" ref="F142" si="14">B142*H142*I142*J142</f>
@@ -3970,12 +3959,12 @@
         <v>1.5</v>
       </c>
       <c r="L142" s="10" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="144" spans="3:12" x14ac:dyDescent="0.2">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="144" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C144" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F144" s="2">
         <f t="shared" ref="F144" si="15">B144*H144*I144*J144</f>
@@ -3991,12 +3980,12 @@
         <v>1.5</v>
       </c>
       <c r="L144" s="10" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="146" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C146" s="2" t="s">
         <v>85</v>
-      </c>
-    </row>
-    <row r="146" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="C146" s="2" t="s">
-        <v>87</v>
       </c>
       <c r="F146" s="2">
         <f t="shared" ref="F146" si="16">B146*H146*I146*J146</f>
@@ -4012,12 +4001,12 @@
         <v>1.5</v>
       </c>
       <c r="L146" s="10" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="148" spans="1:12" x14ac:dyDescent="0.2">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="148" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C148" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="F148" s="2">
         <f t="shared" ref="F148" si="17">B148*H148*I148*J148</f>
@@ -4033,12 +4022,12 @@
         <v>1.5</v>
       </c>
       <c r="L148" s="10" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="150" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="150" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="C150" s="11" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D150" s="11"/>
       <c r="F150" s="2">
@@ -4055,21 +4044,21 @@
         <v>1.5</v>
       </c>
       <c r="L150" s="10" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="152" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="152" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A152" s="1">
         <v>6</v>
       </c>
       <c r="C152" s="3" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D152" s="3"/>
     </row>
-    <row r="154" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C154" s="2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="F154" s="2">
         <f t="shared" ref="F154" si="19">B154*H154*I154*J154</f>
@@ -4085,12 +4074,12 @@
         <v>1.5</v>
       </c>
       <c r="L154" s="10" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="156" spans="1:12" x14ac:dyDescent="0.2">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="156" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C156" s="2" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F156" s="2">
         <f t="shared" ref="F156" si="20">B156*H156*I156*J156</f>
@@ -4106,12 +4095,12 @@
         <v>1.5</v>
       </c>
       <c r="L156" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="158" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C158" s="2" t="s">
         <v>95</v>
-      </c>
-    </row>
-    <row r="158" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="C158" s="2" t="s">
-        <v>97</v>
       </c>
       <c r="F158" s="2">
         <f t="shared" ref="F158" si="21">B158*H158*I158*J158</f>
@@ -4127,12 +4116,12 @@
         <v>1.5</v>
       </c>
       <c r="L158" s="10" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="160" spans="1:12" x14ac:dyDescent="0.2">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="160" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C160" s="2" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F160" s="2">
         <f t="shared" ref="F160" si="22">B160*H160*I160*J160</f>
@@ -4148,12 +4137,12 @@
         <v>1.5</v>
       </c>
       <c r="L160" s="10" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="162" spans="3:12" x14ac:dyDescent="0.2">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="162" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C162" s="2" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F162" s="2">
         <f t="shared" ref="F162" si="23">B162*H162*I162*J162</f>
@@ -4169,12 +4158,12 @@
         <v>1.5</v>
       </c>
       <c r="L162" s="10" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="164" spans="3:12" x14ac:dyDescent="0.2">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="164" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C164" s="2" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F164" s="2">
         <f t="shared" ref="F164" si="24">B164*H164*I164*J164</f>
@@ -4190,12 +4179,12 @@
         <v>1.5</v>
       </c>
       <c r="L164" s="10" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="166" spans="3:12" x14ac:dyDescent="0.2">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="166" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C166" s="2" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F166" s="2">
         <f t="shared" ref="F166" si="25">B166*H166*I166*J166</f>
@@ -4211,12 +4200,12 @@
         <v>1.5</v>
       </c>
       <c r="L166" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="168" spans="3:12" x14ac:dyDescent="0.25">
+      <c r="C168" s="2" t="s">
         <v>101</v>
-      </c>
-    </row>
-    <row r="168" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="C168" s="2" t="s">
-        <v>103</v>
       </c>
       <c r="F168" s="2">
         <f t="shared" ref="F168" si="26">B168*H168*I168*J168</f>
@@ -4232,12 +4221,12 @@
         <v>1.5</v>
       </c>
       <c r="L168" s="10" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="170" spans="3:12" x14ac:dyDescent="0.2">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="170" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C170" s="2" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F170" s="2">
         <f t="shared" ref="F170" si="27">B170*H170*I170*J170</f>
@@ -4253,12 +4242,12 @@
         <v>1.5</v>
       </c>
       <c r="L170" s="10" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="172" spans="3:12" x14ac:dyDescent="0.2">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="172" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C172" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="F172" s="2">
         <f t="shared" ref="F172" si="28">B172*H172*I172*J172</f>
@@ -4274,12 +4263,12 @@
         <v>1.5</v>
       </c>
       <c r="L172" s="10" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="174" spans="3:12" x14ac:dyDescent="0.25">
+      <c r="C174" s="2" t="s">
         <v>106</v>
-      </c>
-    </row>
-    <row r="174" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="C174" s="2" t="s">
-        <v>108</v>
       </c>
       <c r="F174" s="2">
         <f t="shared" ref="F174" si="29">B174*H174*I174*J174</f>
@@ -4295,12 +4284,12 @@
         <v>1.5</v>
       </c>
       <c r="L174" s="10" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="176" spans="3:12" x14ac:dyDescent="0.2">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="176" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C176" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F176" s="2">
         <f t="shared" ref="F176" si="30">B176*H176*I176*J176</f>
@@ -4316,12 +4305,12 @@
         <v>1.5</v>
       </c>
       <c r="L176" s="10" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="178" spans="3:12" x14ac:dyDescent="0.2">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="178" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C178" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="F178" s="2">
         <f t="shared" ref="F178" si="31">B178*H178*I178*J178</f>
@@ -4337,12 +4326,12 @@
         <v>1.5</v>
       </c>
       <c r="L178" s="10" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="180" spans="3:12" x14ac:dyDescent="0.2">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="180" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C180" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F180" s="2">
         <f t="shared" ref="F180" si="32">B180*H180*I180*J180</f>
@@ -4358,12 +4347,12 @@
         <v>1.5</v>
       </c>
       <c r="L180" s="10" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="182" spans="3:12" x14ac:dyDescent="0.2">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="182" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C182" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F182" s="2">
         <f t="shared" ref="F182" si="33">B182*H182*I182*J182</f>
@@ -4379,12 +4368,12 @@
         <v>1.5</v>
       </c>
       <c r="L182" s="10" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="184" spans="3:12" x14ac:dyDescent="0.2">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="184" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C184" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F184" s="2">
         <f t="shared" ref="F184" si="34">B184*H184*I184*J184</f>
@@ -4400,12 +4389,12 @@
         <v>1.5</v>
       </c>
       <c r="L184" s="10" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="186" spans="3:12" x14ac:dyDescent="0.2">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="186" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C186" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="F186" s="2">
         <f t="shared" ref="F186" si="35">B186*H186*I186*J186</f>
@@ -4421,12 +4410,12 @@
         <v>1.5</v>
       </c>
       <c r="L186" s="10" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="188" spans="3:12" x14ac:dyDescent="0.2">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="188" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C188" s="2" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F188" s="2">
         <f t="shared" ref="F188" si="36">B188*H188*I188*J188</f>
@@ -4442,12 +4431,12 @@
         <v>1.5</v>
       </c>
       <c r="L188" s="10" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="190" spans="3:12" x14ac:dyDescent="0.2">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="190" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C190" s="2" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F190" s="2">
         <f t="shared" ref="F190" si="37">B190*H190*I190*J190</f>
@@ -4463,12 +4452,12 @@
         <v>1.5</v>
       </c>
       <c r="L190" s="10" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="192" spans="3:12" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="192" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C192" s="2" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="F192" s="2">
         <f t="shared" ref="F192" si="38">B192*H192*I192*J192</f>
@@ -4484,12 +4473,12 @@
         <v>1.5</v>
       </c>
       <c r="L192" s="10" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="194" spans="1:12" x14ac:dyDescent="0.2">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="194" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C194" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="F194" s="2">
         <f t="shared" ref="F194" si="39">B194*H194*I194*J194</f>
@@ -4505,12 +4494,12 @@
         <v>1.5</v>
       </c>
       <c r="L194" s="10" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="196" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C196" s="2" t="s">
         <v>121</v>
-      </c>
-    </row>
-    <row r="196" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="C196" s="2" t="s">
-        <v>123</v>
       </c>
       <c r="F196" s="2">
         <f t="shared" ref="F196" si="40">B196*H196*I196*J196</f>
@@ -4526,12 +4515,12 @@
         <v>1.5</v>
       </c>
       <c r="L196" s="10" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="198" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C198" s="2" t="s">
         <v>121</v>
-      </c>
-    </row>
-    <row r="198" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="C198" s="2" t="s">
-        <v>123</v>
       </c>
       <c r="F198" s="2">
         <f t="shared" ref="F198" si="41">B198*H198*I198*J198</f>
@@ -4547,12 +4536,12 @@
         <v>1.5</v>
       </c>
       <c r="L198" s="10" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="200" spans="1:12" x14ac:dyDescent="0.2">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="200" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C200" s="2" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="F200" s="2">
         <f t="shared" ref="F200" si="42">B200*H200*I200*J200</f>
@@ -4568,12 +4557,12 @@
         <v>1.5</v>
       </c>
       <c r="L200" s="10" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="202" spans="1:12" x14ac:dyDescent="0.2">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="202" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C202" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="F202" s="2">
         <f t="shared" ref="F202" si="43">B202*H202*I202*J202</f>
@@ -4589,21 +4578,21 @@
         <v>1.5</v>
       </c>
       <c r="L202" s="10" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="206" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="206" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A206" s="1">
         <v>7</v>
       </c>
       <c r="C206" s="3" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="D206" s="3"/>
     </row>
-    <row r="208" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C208" s="2" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="F208" s="2">
         <f t="shared" ref="F208" si="44">B208*H208*I208*J208</f>
@@ -4619,15 +4608,15 @@
         <v>1.5</v>
       </c>
       <c r="L208" s="10" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="209" spans="1:12" x14ac:dyDescent="0.2">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="209" spans="1:12" ht="16.3" x14ac:dyDescent="0.3">
       <c r="E209"/>
     </row>
-    <row r="210" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C210" s="2" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="F210" s="2">
         <f t="shared" ref="F210" si="45">B210*H210*I210*J210</f>
@@ -4643,12 +4632,12 @@
         <v>1.5</v>
       </c>
       <c r="L210" s="10" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="212" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C212" s="2" t="s">
         <v>130</v>
-      </c>
-    </row>
-    <row r="212" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="C212" s="2" t="s">
-        <v>132</v>
       </c>
       <c r="F212" s="2">
         <f t="shared" ref="F212" si="46">B212*H212*I212*J212</f>
@@ -4664,12 +4653,12 @@
         <v>1.5</v>
       </c>
       <c r="L212" s="10" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="214" spans="1:12" x14ac:dyDescent="0.2">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="214" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C214" s="2" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="F214" s="2">
         <f t="shared" ref="F214" si="47">B214*H214*I214*J214</f>
@@ -4685,12 +4674,12 @@
         <v>1.5</v>
       </c>
       <c r="L214" s="10" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="216" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C216" s="2" t="s">
         <v>133</v>
-      </c>
-    </row>
-    <row r="216" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="C216" s="2" t="s">
-        <v>135</v>
       </c>
       <c r="F216" s="2">
         <f t="shared" ref="F216" si="48">B216*H216*I216*J216</f>
@@ -4706,12 +4695,12 @@
         <v>1.5</v>
       </c>
       <c r="L216" s="10" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="218" spans="1:12" x14ac:dyDescent="0.2">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="218" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C218" s="2" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F218" s="2">
         <f t="shared" ref="F218" si="49">B218*H218*I218*J218</f>
@@ -4727,12 +4716,12 @@
         <v>1.5</v>
       </c>
       <c r="L218" s="10" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="220" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C220" s="2" t="s">
         <v>136</v>
-      </c>
-    </row>
-    <row r="220" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="C220" s="2" t="s">
-        <v>138</v>
       </c>
       <c r="F220" s="2">
         <f t="shared" ref="F220" si="50">B220*H220*I220*J220</f>
@@ -4748,21 +4737,21 @@
         <v>1.5</v>
       </c>
       <c r="L220" s="10" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="223" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="223" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A223" s="1">
         <v>8</v>
       </c>
       <c r="C223" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D223" s="3"/>
     </row>
-    <row r="225" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C225" s="2" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="F225" s="2">
         <f t="shared" ref="F225" si="51">B225*H225*I225*J225</f>
@@ -4778,12 +4767,12 @@
         <v>1.5</v>
       </c>
       <c r="L225" s="10" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="227" spans="1:12" x14ac:dyDescent="0.2">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="227" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C227" s="2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="F227" s="2">
         <f t="shared" ref="F227" si="52">B227*H227*I227*J227</f>
@@ -4799,12 +4788,12 @@
         <v>1.5</v>
       </c>
       <c r="L227" s="10" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="229" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C229" s="2" t="s">
         <v>142</v>
-      </c>
-    </row>
-    <row r="229" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="C229" s="2" t="s">
-        <v>144</v>
       </c>
       <c r="F229" s="2">
         <f t="shared" ref="F229" si="53">B229*H229*I229*J229</f>
@@ -4820,12 +4809,12 @@
         <v>1.5</v>
       </c>
       <c r="L229" s="10" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="231" spans="1:12" x14ac:dyDescent="0.2">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="231" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C231" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="F231" s="2">
         <f t="shared" ref="F231" si="54">B231*H231*I231*J231</f>
@@ -4841,21 +4830,21 @@
         <v>1.5</v>
       </c>
       <c r="L231" s="10" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="236" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="236" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A236" s="1">
         <v>9</v>
       </c>
       <c r="C236" s="3" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D236" s="3"/>
     </row>
-    <row r="238" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C238" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F238" s="2">
         <f t="shared" ref="F238" si="55">B238*H238*I238*J238</f>
@@ -4871,12 +4860,12 @@
         <v>1.5</v>
       </c>
       <c r="L238" s="10" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="240" spans="1:12" x14ac:dyDescent="0.2">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="240" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C240" s="2" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F240" s="2">
         <f t="shared" ref="F240" si="56">B240*H240*I240*J240</f>
@@ -4892,17 +4881,17 @@
         <v>1.5</v>
       </c>
       <c r="L240" s="10" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="241" spans="3:12" x14ac:dyDescent="0.25">
+      <c r="L241" s="10" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="243" spans="3:12" x14ac:dyDescent="0.25">
+      <c r="C243" s="2" t="s">
         <v>150</v>
-      </c>
-    </row>
-    <row r="241" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="L241" s="10" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="243" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="C243" s="2" t="s">
-        <v>152</v>
       </c>
       <c r="F243" s="2">
         <f t="shared" ref="F243" si="57">B243*H243*I243*J243</f>
@@ -4918,12 +4907,12 @@
         <v>1.5</v>
       </c>
       <c r="L243" s="10" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="245" spans="3:12" x14ac:dyDescent="0.2">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="245" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C245" s="2" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="F245" s="2">
         <f t="shared" ref="F245" si="58">B245*H245*I245*J245</f>
@@ -4939,12 +4928,12 @@
         <v>1.5</v>
       </c>
       <c r="L245" s="10" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="247" spans="3:12" x14ac:dyDescent="0.2">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="247" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C247" s="2" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="F247" s="2">
         <f t="shared" ref="F247" si="59">B247*H247*I247*J247</f>
@@ -4960,17 +4949,17 @@
         <v>1.5</v>
       </c>
       <c r="L247" s="10" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="248" spans="3:12" x14ac:dyDescent="0.2">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="248" spans="3:12" x14ac:dyDescent="0.25">
       <c r="L248" s="10" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="250" spans="3:12" x14ac:dyDescent="0.2">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="250" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C250" s="2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="F250" s="2">
         <f>B250*H250*I250*J250</f>
@@ -4986,17 +4975,17 @@
         <v>1.5</v>
       </c>
       <c r="L250" s="10" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="251" spans="3:12" x14ac:dyDescent="0.25">
+      <c r="L251" s="10" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="253" spans="3:12" x14ac:dyDescent="0.25">
+      <c r="C253" s="2" t="s">
         <v>156</v>
-      </c>
-    </row>
-    <row r="251" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="L251" s="10" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="253" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="C253" s="2" t="s">
-        <v>158</v>
       </c>
       <c r="F253" s="2">
         <f t="shared" ref="F253" si="60">B253*H253*I253*J253</f>
@@ -5012,12 +5001,12 @@
         <v>1.5</v>
       </c>
       <c r="L253" s="10" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="255" spans="3:12" x14ac:dyDescent="0.2">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="255" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C255" s="2" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="F255" s="2">
         <f t="shared" ref="F255" si="61">B255*H255*I255*J255</f>
@@ -5033,12 +5022,12 @@
         <v>1.5</v>
       </c>
       <c r="L255" s="10" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="257" spans="1:12" x14ac:dyDescent="0.2">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="257" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C257" s="2" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="F257" s="2">
         <f t="shared" ref="F257" si="62">B257*H257*I257*J257</f>
@@ -5054,17 +5043,17 @@
         <v>1.5</v>
       </c>
       <c r="L257" s="10" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="258" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C258" s="2" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="260" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C260" s="2" t="s">
         <v>163</v>
-      </c>
-    </row>
-    <row r="258" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="C258" s="2" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="260" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="C260" s="2" t="s">
-        <v>165</v>
       </c>
       <c r="F260" s="2">
         <f t="shared" ref="F260" si="63">B260*H260*I260*J260</f>
@@ -5080,17 +5069,17 @@
         <v>1.5</v>
       </c>
       <c r="L260" s="10" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="261" spans="1:12" x14ac:dyDescent="0.2">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="261" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C261" s="2" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="263" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="263" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="C263" s="12" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="D263" s="12"/>
       <c r="F263" s="2">
@@ -5107,21 +5096,21 @@
         <v>1.5</v>
       </c>
       <c r="L263" s="10" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="266" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="266" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A266" s="1">
         <v>10</v>
       </c>
       <c r="C266" s="3" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="D266" s="3"/>
     </row>
-    <row r="268" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="268" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C268" s="2" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="F268" s="2">
         <f t="shared" ref="F268" si="65">B268*H268*I268*J268</f>
@@ -5137,12 +5126,12 @@
         <v>1.2</v>
       </c>
       <c r="L268" s="10" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="270" spans="1:12" x14ac:dyDescent="0.2">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="270" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C270" s="2" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="F270" s="2">
         <f t="shared" ref="F270" si="66">B270*H270*I270*J270</f>
@@ -5158,20 +5147,20 @@
         <v>1.2</v>
       </c>
       <c r="L270" s="10" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="274" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="274" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A274" s="1">
         <v>11</v>
       </c>
       <c r="C274" s="13" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="276" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="276" spans="1:12" ht="17" x14ac:dyDescent="0.3">
       <c r="C276" s="12" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D276" s="14"/>
       <c r="E276" s="15"/>
@@ -5189,17 +5178,17 @@
         <v>1.5</v>
       </c>
       <c r="L276" s="10" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="277" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="277" spans="1:12" ht="17" x14ac:dyDescent="0.3">
       <c r="C277" s="12"/>
       <c r="D277" s="14"/>
       <c r="E277" s="15"/>
     </row>
-    <row r="278" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="278" spans="1:12" ht="17" x14ac:dyDescent="0.3">
       <c r="C278" s="12" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D278" s="14"/>
       <c r="E278" s="15"/>
@@ -5217,7 +5206,7 @@
         <v>1.5</v>
       </c>
       <c r="L278" s="10" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix pricing import flow, basis review state, and CI checks (#15)
* Fix pricing import and basis review flows

* Harden pricing references and polish quote basis UI

* Refactor quote generation workflow and layout handling

* Add pricing catalog image extraction and fix output row matching

* Fix CI basis chat smoke flow

* Fix CI security gates
</commit_message>
<xml_diff>
--- a/docs/Quotation-Cost-Template-V1.1.xlsx
+++ b/docs/Quotation-Cost-Template-V1.1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aaa/Konceptliving Dropbox/Konceptliving Team Folder/KONCEPT QUOTATION/Template/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\xPass\GitHub Projects\koncept-quote-auto-generator\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB79C0DD-FACC-494E-8BC4-640909092A90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49393CF8-8C7E-48F1-AF17-D06C518ACAEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="25600" windowHeight="14040" xr2:uid="{C830D79F-9B19-7342-9B39-F4DE5434FDDB}"/>
+    <workbookView xWindow="-109" yWindow="-109" windowWidth="26301" windowHeight="14169" xr2:uid="{C830D79F-9B19-7342-9B39-F4DE5434FDDB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -19,17 +19,6 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -395,15 +384,9 @@
     <t>HQI Floodlight</t>
   </si>
   <si>
-    <t>nos. LED recess dowlight 3"</t>
-  </si>
-  <si>
     <t>Downlight</t>
   </si>
   <si>
-    <t>nos. LED recess dowlight 6"</t>
-  </si>
-  <si>
     <t>nos.13Amp/230V SP 50Hz AC Socket (Max 800W) (Not for lighting use) </t>
   </si>
   <si>
@@ -702,6 +685,12 @@
   </si>
   <si>
     <t>COFFEE PER DAY</t>
+  </si>
+  <si>
+    <t>nos. LED recess downlight 3"</t>
+  </si>
+  <si>
+    <t>nos. LED recess downlight 6"</t>
   </si>
 </sst>
 </file>
@@ -2691,18 +2680,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2355A233-406B-9740-B1B1-24942A627A7E}">
   <dimension ref="A2:O278"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.77734375" defaultRowHeight="15.65" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="10.83203125" style="2"/>
+    <col min="1" max="2" width="10.77734375" style="2"/>
     <col min="3" max="3" width="44.33203125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="18.77734375" style="2" customWidth="1"/>
     <col min="5" max="5" width="13" style="2" customWidth="1"/>
-    <col min="6" max="11" width="10.83203125" style="2"/>
+    <col min="6" max="11" width="10.77734375" style="2"/>
     <col min="12" max="12" width="25.33203125" style="10" customWidth="1"/>
-    <col min="13" max="16384" width="10.83203125" style="2"/>
+    <col min="13" max="16384" width="10.77734375" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="5">
         <v>1</v>
       </c>
@@ -2727,7 +2716,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="18" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12" ht="18.350000000000001" x14ac:dyDescent="0.25">
       <c r="C4" s="8" t="s">
         <v>6</v>
       </c>
@@ -2749,7 +2738,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="18" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:12" ht="18.350000000000001" x14ac:dyDescent="0.25">
       <c r="C6" s="8" t="s">
         <v>8</v>
       </c>
@@ -2771,7 +2760,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="18" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:12" ht="18.350000000000001" x14ac:dyDescent="0.25">
       <c r="C8" s="8" t="s">
         <v>10</v>
       </c>
@@ -2793,7 +2782,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="18" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:12" ht="18.350000000000001" x14ac:dyDescent="0.25">
       <c r="C10" s="8" t="s">
         <v>12</v>
       </c>
@@ -2815,7 +2804,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="18" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:12" ht="18.350000000000001" x14ac:dyDescent="0.25">
       <c r="C12" s="8" t="s">
         <v>14</v>
       </c>
@@ -2837,7 +2826,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="18" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:12" ht="18.350000000000001" x14ac:dyDescent="0.25">
       <c r="C14" s="8" t="s">
         <v>16</v>
       </c>
@@ -2859,7 +2848,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>2</v>
       </c>
@@ -2868,9 +2857,9 @@
       </c>
       <c r="D17" s="3"/>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C19" s="2" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="F19" s="2">
         <f>B19*H19*J19</f>
@@ -2886,7 +2875,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C20" s="2" t="s">
         <v>20</v>
       </c>
@@ -2894,9 +2883,9 @@
         <v>21</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C22" s="2" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="F22" s="2">
         <f>B22*H22*J22</f>
@@ -2912,7 +2901,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C23" s="2" t="s">
         <v>31</v>
       </c>
@@ -2920,9 +2909,9 @@
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C25" s="2" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F25" s="2">
         <f>B25*H25*J25</f>
@@ -2938,7 +2927,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C26" s="2" t="s">
         <v>25</v>
       </c>
@@ -2946,9 +2935,9 @@
         <v>21</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C28" s="2" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F28" s="2">
         <f>B28*H28*J28</f>
@@ -2964,7 +2953,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C29" s="2" t="s">
         <v>22</v>
       </c>
@@ -2972,7 +2961,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C31" s="2" t="s">
         <v>27</v>
       </c>
@@ -2990,7 +2979,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C32" s="2" t="s">
         <v>20</v>
       </c>
@@ -2998,7 +2987,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="34" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="34" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C34" s="2" t="s">
         <v>27</v>
       </c>
@@ -3016,7 +3005,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="35" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="35" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C35" s="2" t="s">
         <v>22</v>
       </c>
@@ -3024,7 +3013,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="37" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="37" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C37" s="2" t="s">
         <v>28</v>
       </c>
@@ -3042,7 +3031,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="38" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="38" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C38" s="2" t="s">
         <v>20</v>
       </c>
@@ -3050,7 +3039,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="40" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="40" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C40" s="2" t="s">
         <v>28</v>
       </c>
@@ -3068,7 +3057,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="41" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="41" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C41" s="2" t="s">
         <v>22</v>
       </c>
@@ -3076,7 +3065,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="44" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="44" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C44" s="2" t="s">
         <v>29</v>
       </c>
@@ -3094,7 +3083,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="45" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="45" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C45" s="2" t="s">
         <v>20</v>
       </c>
@@ -3102,7 +3091,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="47" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="47" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C47" s="2" t="s">
         <v>29</v>
       </c>
@@ -3120,7 +3109,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="48" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="48" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C48" s="2" t="s">
         <v>31</v>
       </c>
@@ -3128,7 +3117,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="50" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="50" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C50" s="2" t="s">
         <v>32</v>
       </c>
@@ -3146,7 +3135,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="51" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="51" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C51" s="2" t="s">
         <v>20</v>
       </c>
@@ -3154,7 +3143,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="53" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="53" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C53" s="2" t="s">
         <v>32</v>
       </c>
@@ -3172,7 +3161,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="54" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="54" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C54" s="2" t="s">
         <v>31</v>
       </c>
@@ -3180,7 +3169,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="56" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="56" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C56" s="2" t="s">
         <v>34</v>
       </c>
@@ -3198,12 +3187,12 @@
         <v>35</v>
       </c>
     </row>
-    <row r="57" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="57" spans="3:12" x14ac:dyDescent="0.25">
       <c r="L57" s="10" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="59" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="59" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C59" s="2" t="s">
         <v>36</v>
       </c>
@@ -3221,14 +3210,14 @@
         <v>35</v>
       </c>
     </row>
-    <row r="60" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="60" spans="3:12" x14ac:dyDescent="0.25">
       <c r="L60" s="10" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="62" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="62" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C62" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="F62" s="2">
         <f>B62*H62*J62</f>
@@ -3242,15 +3231,15 @@
         <v>1.5</v>
       </c>
       <c r="L62" s="10" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="63" spans="3:12" x14ac:dyDescent="0.2">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="63" spans="3:12" x14ac:dyDescent="0.25">
       <c r="L63" s="10" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="65" spans="3:12" x14ac:dyDescent="0.2">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="65" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C65" s="2" t="s">
         <v>37</v>
       </c>
@@ -3268,12 +3257,12 @@
         <v>38</v>
       </c>
     </row>
-    <row r="66" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="66" spans="3:12" x14ac:dyDescent="0.25">
       <c r="L66" s="10" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="68" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="68" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C68" s="2" t="s">
         <v>39</v>
       </c>
@@ -3291,12 +3280,12 @@
         <v>38</v>
       </c>
     </row>
-    <row r="69" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="69" spans="3:12" x14ac:dyDescent="0.25">
       <c r="L69" s="10" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="71" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="71" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C71" s="2" t="s">
         <v>40</v>
       </c>
@@ -3314,12 +3303,12 @@
         <v>41</v>
       </c>
     </row>
-    <row r="72" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="72" spans="3:12" x14ac:dyDescent="0.25">
       <c r="L72" s="10" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="74" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="74" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C74" s="2" t="s">
         <v>42</v>
       </c>
@@ -3337,12 +3326,12 @@
         <v>41</v>
       </c>
     </row>
-    <row r="75" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="75" spans="3:12" x14ac:dyDescent="0.25">
       <c r="L75" s="10" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="77" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="77" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C77" s="2" t="s">
         <v>43</v>
       </c>
@@ -3360,7 +3349,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="81" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A81" s="1">
         <v>3</v>
       </c>
@@ -3369,12 +3358,12 @@
       </c>
       <c r="D81" s="3"/>
     </row>
-    <row r="82" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A82" s="1"/>
       <c r="C82" s="3"/>
       <c r="D82" s="3"/>
     </row>
-    <row r="83" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A83" s="1"/>
       <c r="C83" s="2" t="s">
         <v>46</v>
@@ -3393,7 +3382,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="84" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A84" s="1"/>
       <c r="C84" s="2" t="s">
         <v>48</v>
@@ -3402,10 +3391,10 @@
         <v>21</v>
       </c>
     </row>
-    <row r="85" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A85" s="1"/>
     </row>
-    <row r="86" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A86" s="1"/>
       <c r="C86" s="2" t="s">
         <v>46</v>
@@ -3424,7 +3413,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="87" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A87" s="1"/>
       <c r="C87" s="2" t="s">
         <v>31</v>
@@ -3433,10 +3422,10 @@
         <v>49</v>
       </c>
     </row>
-    <row r="88" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A88" s="1"/>
     </row>
-    <row r="89" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A89" s="1"/>
       <c r="C89" s="2" t="s">
         <v>50</v>
@@ -3455,7 +3444,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="90" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A90" s="1"/>
       <c r="C90" s="2" t="s">
         <v>48</v>
@@ -3464,10 +3453,10 @@
         <v>21</v>
       </c>
     </row>
-    <row r="91" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A91" s="1"/>
     </row>
-    <row r="92" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A92" s="1"/>
       <c r="C92" s="2" t="s">
         <v>50</v>
@@ -3486,7 +3475,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="93" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A93" s="1"/>
       <c r="C93" s="2" t="s">
         <v>31</v>
@@ -3495,10 +3484,10 @@
         <v>49</v>
       </c>
     </row>
-    <row r="94" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A94" s="1"/>
     </row>
-    <row r="95" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A95" s="1"/>
       <c r="C95" s="2" t="s">
         <v>52</v>
@@ -3517,7 +3506,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="96" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A96" s="1"/>
       <c r="C96" s="2" t="s">
         <v>48</v>
@@ -3526,10 +3515,10 @@
         <v>21</v>
       </c>
     </row>
-    <row r="97" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A97" s="1"/>
     </row>
-    <row r="98" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A98" s="1"/>
       <c r="C98" s="2" t="s">
         <v>52</v>
@@ -3548,7 +3537,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="99" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A99" s="1"/>
       <c r="C99" s="2" t="s">
         <v>31</v>
@@ -3557,10 +3546,10 @@
         <v>49</v>
       </c>
     </row>
-    <row r="100" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A100" s="1"/>
     </row>
-    <row r="101" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A101" s="1"/>
       <c r="C101" s="2" t="s">
         <v>54</v>
@@ -3582,10 +3571,10 @@
         <v>55</v>
       </c>
     </row>
-    <row r="102" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A102" s="1"/>
     </row>
-    <row r="104" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A104" s="1">
         <v>4</v>
       </c>
@@ -3594,7 +3583,7 @@
       </c>
       <c r="D104" s="3"/>
     </row>
-    <row r="106" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C106" s="2" t="s">
         <v>57</v>
       </c>
@@ -3615,7 +3604,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="108" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C108" s="2" t="s">
         <v>59</v>
       </c>
@@ -3636,16 +3625,16 @@
         <v>60</v>
       </c>
     </row>
-    <row r="109" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C109" s="2" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="110" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C110" s="4"/>
       <c r="D110" s="4"/>
     </row>
-    <row r="111" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C111" s="2" t="s">
         <v>62</v>
       </c>
@@ -3666,7 +3655,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="113" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B113" s="2">
         <v>1</v>
       </c>
@@ -3690,7 +3679,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="115" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C115" s="2" t="s">
         <v>66</v>
       </c>
@@ -3711,7 +3700,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="116" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C116" s="2" t="s">
         <v>20</v>
       </c>
@@ -3719,7 +3708,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="118" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C118" s="2" t="s">
         <v>66</v>
       </c>
@@ -3740,7 +3729,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="119" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C119" s="2" t="s">
         <v>31</v>
       </c>
@@ -3748,7 +3737,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="121" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C121" s="2" t="s">
         <v>66</v>
       </c>
@@ -3769,17 +3758,17 @@
         <v>68</v>
       </c>
     </row>
-    <row r="122" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C122" s="2" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="123" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C123" s="2" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="125" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C125" s="2" t="s">
         <v>71</v>
       </c>
@@ -3808,7 +3797,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="126" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:15" x14ac:dyDescent="0.25">
       <c r="N126" s="2">
         <v>1000</v>
       </c>
@@ -3817,7 +3806,7 @@
         <v>14.705882352941176</v>
       </c>
     </row>
-    <row r="128" spans="1:15" ht="17" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:15" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A128" s="1">
         <v>5</v>
       </c>
@@ -3826,7 +3815,7 @@
       </c>
       <c r="D128" s="3"/>
     </row>
-    <row r="130" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="130" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C130" s="2" t="s">
         <v>73</v>
       </c>
@@ -3847,7 +3836,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="132" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="132" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C132" s="2" t="s">
         <v>75</v>
       </c>
@@ -3868,7 +3857,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="134" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="134" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C134" s="2" t="s">
         <v>77</v>
       </c>
@@ -3889,7 +3878,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="136" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="136" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C136" s="2" t="s">
         <v>79</v>
       </c>
@@ -3910,9 +3899,9 @@
         <v>80</v>
       </c>
     </row>
-    <row r="138" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="138" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C138" s="2" t="s">
-        <v>81</v>
+        <v>182</v>
       </c>
       <c r="F138" s="2">
         <f t="shared" ref="F138" si="12">B138*H138*I138*J138</f>
@@ -3928,12 +3917,12 @@
         <v>1.5</v>
       </c>
       <c r="L138" s="10" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="140" spans="3:12" x14ac:dyDescent="0.2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="140" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C140" s="2" t="s">
-        <v>83</v>
+        <v>183</v>
       </c>
       <c r="F140" s="2">
         <f t="shared" ref="F140" si="13">B140*H140*I140*J140</f>
@@ -3949,12 +3938,12 @@
         <v>1.5</v>
       </c>
       <c r="L140" s="10" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="142" spans="3:12" x14ac:dyDescent="0.25">
+      <c r="C142" s="2" t="s">
         <v>82</v>
-      </c>
-    </row>
-    <row r="142" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="C142" s="2" t="s">
-        <v>84</v>
       </c>
       <c r="F142" s="2">
         <f t="shared" ref="F142" si="14">B142*H142*I142*J142</f>
@@ -3970,12 +3959,12 @@
         <v>1.5</v>
       </c>
       <c r="L142" s="10" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="144" spans="3:12" x14ac:dyDescent="0.2">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="144" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C144" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F144" s="2">
         <f t="shared" ref="F144" si="15">B144*H144*I144*J144</f>
@@ -3991,12 +3980,12 @@
         <v>1.5</v>
       </c>
       <c r="L144" s="10" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="146" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C146" s="2" t="s">
         <v>85</v>
-      </c>
-    </row>
-    <row r="146" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="C146" s="2" t="s">
-        <v>87</v>
       </c>
       <c r="F146" s="2">
         <f t="shared" ref="F146" si="16">B146*H146*I146*J146</f>
@@ -4012,12 +4001,12 @@
         <v>1.5</v>
       </c>
       <c r="L146" s="10" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="148" spans="1:12" x14ac:dyDescent="0.2">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="148" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C148" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="F148" s="2">
         <f t="shared" ref="F148" si="17">B148*H148*I148*J148</f>
@@ -4033,12 +4022,12 @@
         <v>1.5</v>
       </c>
       <c r="L148" s="10" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="150" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="150" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="C150" s="11" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D150" s="11"/>
       <c r="F150" s="2">
@@ -4055,21 +4044,21 @@
         <v>1.5</v>
       </c>
       <c r="L150" s="10" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="152" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="152" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A152" s="1">
         <v>6</v>
       </c>
       <c r="C152" s="3" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D152" s="3"/>
     </row>
-    <row r="154" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C154" s="2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="F154" s="2">
         <f t="shared" ref="F154" si="19">B154*H154*I154*J154</f>
@@ -4085,12 +4074,12 @@
         <v>1.5</v>
       </c>
       <c r="L154" s="10" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="156" spans="1:12" x14ac:dyDescent="0.2">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="156" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C156" s="2" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F156" s="2">
         <f t="shared" ref="F156" si="20">B156*H156*I156*J156</f>
@@ -4106,12 +4095,12 @@
         <v>1.5</v>
       </c>
       <c r="L156" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="158" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C158" s="2" t="s">
         <v>95</v>
-      </c>
-    </row>
-    <row r="158" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="C158" s="2" t="s">
-        <v>97</v>
       </c>
       <c r="F158" s="2">
         <f t="shared" ref="F158" si="21">B158*H158*I158*J158</f>
@@ -4127,12 +4116,12 @@
         <v>1.5</v>
       </c>
       <c r="L158" s="10" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="160" spans="1:12" x14ac:dyDescent="0.2">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="160" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C160" s="2" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F160" s="2">
         <f t="shared" ref="F160" si="22">B160*H160*I160*J160</f>
@@ -4148,12 +4137,12 @@
         <v>1.5</v>
       </c>
       <c r="L160" s="10" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="162" spans="3:12" x14ac:dyDescent="0.2">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="162" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C162" s="2" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F162" s="2">
         <f t="shared" ref="F162" si="23">B162*H162*I162*J162</f>
@@ -4169,12 +4158,12 @@
         <v>1.5</v>
       </c>
       <c r="L162" s="10" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="164" spans="3:12" x14ac:dyDescent="0.2">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="164" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C164" s="2" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F164" s="2">
         <f t="shared" ref="F164" si="24">B164*H164*I164*J164</f>
@@ -4190,12 +4179,12 @@
         <v>1.5</v>
       </c>
       <c r="L164" s="10" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="166" spans="3:12" x14ac:dyDescent="0.2">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="166" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C166" s="2" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F166" s="2">
         <f t="shared" ref="F166" si="25">B166*H166*I166*J166</f>
@@ -4211,12 +4200,12 @@
         <v>1.5</v>
       </c>
       <c r="L166" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="168" spans="3:12" x14ac:dyDescent="0.25">
+      <c r="C168" s="2" t="s">
         <v>101</v>
-      </c>
-    </row>
-    <row r="168" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="C168" s="2" t="s">
-        <v>103</v>
       </c>
       <c r="F168" s="2">
         <f t="shared" ref="F168" si="26">B168*H168*I168*J168</f>
@@ -4232,12 +4221,12 @@
         <v>1.5</v>
       </c>
       <c r="L168" s="10" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="170" spans="3:12" x14ac:dyDescent="0.2">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="170" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C170" s="2" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F170" s="2">
         <f t="shared" ref="F170" si="27">B170*H170*I170*J170</f>
@@ -4253,12 +4242,12 @@
         <v>1.5</v>
       </c>
       <c r="L170" s="10" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="172" spans="3:12" x14ac:dyDescent="0.2">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="172" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C172" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="F172" s="2">
         <f t="shared" ref="F172" si="28">B172*H172*I172*J172</f>
@@ -4274,12 +4263,12 @@
         <v>1.5</v>
       </c>
       <c r="L172" s="10" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="174" spans="3:12" x14ac:dyDescent="0.25">
+      <c r="C174" s="2" t="s">
         <v>106</v>
-      </c>
-    </row>
-    <row r="174" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="C174" s="2" t="s">
-        <v>108</v>
       </c>
       <c r="F174" s="2">
         <f t="shared" ref="F174" si="29">B174*H174*I174*J174</f>
@@ -4295,12 +4284,12 @@
         <v>1.5</v>
       </c>
       <c r="L174" s="10" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="176" spans="3:12" x14ac:dyDescent="0.2">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="176" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C176" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F176" s="2">
         <f t="shared" ref="F176" si="30">B176*H176*I176*J176</f>
@@ -4316,12 +4305,12 @@
         <v>1.5</v>
       </c>
       <c r="L176" s="10" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="178" spans="3:12" x14ac:dyDescent="0.2">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="178" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C178" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="F178" s="2">
         <f t="shared" ref="F178" si="31">B178*H178*I178*J178</f>
@@ -4337,12 +4326,12 @@
         <v>1.5</v>
       </c>
       <c r="L178" s="10" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="180" spans="3:12" x14ac:dyDescent="0.2">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="180" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C180" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F180" s="2">
         <f t="shared" ref="F180" si="32">B180*H180*I180*J180</f>
@@ -4358,12 +4347,12 @@
         <v>1.5</v>
       </c>
       <c r="L180" s="10" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="182" spans="3:12" x14ac:dyDescent="0.2">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="182" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C182" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F182" s="2">
         <f t="shared" ref="F182" si="33">B182*H182*I182*J182</f>
@@ -4379,12 +4368,12 @@
         <v>1.5</v>
       </c>
       <c r="L182" s="10" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="184" spans="3:12" x14ac:dyDescent="0.2">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="184" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C184" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F184" s="2">
         <f t="shared" ref="F184" si="34">B184*H184*I184*J184</f>
@@ -4400,12 +4389,12 @@
         <v>1.5</v>
       </c>
       <c r="L184" s="10" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="186" spans="3:12" x14ac:dyDescent="0.2">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="186" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C186" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="F186" s="2">
         <f t="shared" ref="F186" si="35">B186*H186*I186*J186</f>
@@ -4421,12 +4410,12 @@
         <v>1.5</v>
       </c>
       <c r="L186" s="10" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="188" spans="3:12" x14ac:dyDescent="0.2">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="188" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C188" s="2" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F188" s="2">
         <f t="shared" ref="F188" si="36">B188*H188*I188*J188</f>
@@ -4442,12 +4431,12 @@
         <v>1.5</v>
       </c>
       <c r="L188" s="10" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="190" spans="3:12" x14ac:dyDescent="0.2">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="190" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C190" s="2" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F190" s="2">
         <f t="shared" ref="F190" si="37">B190*H190*I190*J190</f>
@@ -4463,12 +4452,12 @@
         <v>1.5</v>
       </c>
       <c r="L190" s="10" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="192" spans="3:12" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="192" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C192" s="2" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="F192" s="2">
         <f t="shared" ref="F192" si="38">B192*H192*I192*J192</f>
@@ -4484,12 +4473,12 @@
         <v>1.5</v>
       </c>
       <c r="L192" s="10" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="194" spans="1:12" x14ac:dyDescent="0.2">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="194" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C194" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="F194" s="2">
         <f t="shared" ref="F194" si="39">B194*H194*I194*J194</f>
@@ -4505,12 +4494,12 @@
         <v>1.5</v>
       </c>
       <c r="L194" s="10" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="196" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C196" s="2" t="s">
         <v>121</v>
-      </c>
-    </row>
-    <row r="196" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="C196" s="2" t="s">
-        <v>123</v>
       </c>
       <c r="F196" s="2">
         <f t="shared" ref="F196" si="40">B196*H196*I196*J196</f>
@@ -4526,12 +4515,12 @@
         <v>1.5</v>
       </c>
       <c r="L196" s="10" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="198" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C198" s="2" t="s">
         <v>121</v>
-      </c>
-    </row>
-    <row r="198" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="C198" s="2" t="s">
-        <v>123</v>
       </c>
       <c r="F198" s="2">
         <f t="shared" ref="F198" si="41">B198*H198*I198*J198</f>
@@ -4547,12 +4536,12 @@
         <v>1.5</v>
       </c>
       <c r="L198" s="10" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="200" spans="1:12" x14ac:dyDescent="0.2">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="200" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C200" s="2" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="F200" s="2">
         <f t="shared" ref="F200" si="42">B200*H200*I200*J200</f>
@@ -4568,12 +4557,12 @@
         <v>1.5</v>
       </c>
       <c r="L200" s="10" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="202" spans="1:12" x14ac:dyDescent="0.2">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="202" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C202" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="F202" s="2">
         <f t="shared" ref="F202" si="43">B202*H202*I202*J202</f>
@@ -4589,21 +4578,21 @@
         <v>1.5</v>
       </c>
       <c r="L202" s="10" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="206" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="206" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A206" s="1">
         <v>7</v>
       </c>
       <c r="C206" s="3" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="D206" s="3"/>
     </row>
-    <row r="208" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C208" s="2" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="F208" s="2">
         <f t="shared" ref="F208" si="44">B208*H208*I208*J208</f>
@@ -4619,15 +4608,15 @@
         <v>1.5</v>
       </c>
       <c r="L208" s="10" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="209" spans="1:12" x14ac:dyDescent="0.2">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="209" spans="1:12" ht="16.3" x14ac:dyDescent="0.3">
       <c r="E209"/>
     </row>
-    <row r="210" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C210" s="2" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="F210" s="2">
         <f t="shared" ref="F210" si="45">B210*H210*I210*J210</f>
@@ -4643,12 +4632,12 @@
         <v>1.5</v>
       </c>
       <c r="L210" s="10" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="212" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C212" s="2" t="s">
         <v>130</v>
-      </c>
-    </row>
-    <row r="212" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="C212" s="2" t="s">
-        <v>132</v>
       </c>
       <c r="F212" s="2">
         <f t="shared" ref="F212" si="46">B212*H212*I212*J212</f>
@@ -4664,12 +4653,12 @@
         <v>1.5</v>
       </c>
       <c r="L212" s="10" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="214" spans="1:12" x14ac:dyDescent="0.2">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="214" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C214" s="2" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="F214" s="2">
         <f t="shared" ref="F214" si="47">B214*H214*I214*J214</f>
@@ -4685,12 +4674,12 @@
         <v>1.5</v>
       </c>
       <c r="L214" s="10" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="216" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C216" s="2" t="s">
         <v>133</v>
-      </c>
-    </row>
-    <row r="216" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="C216" s="2" t="s">
-        <v>135</v>
       </c>
       <c r="F216" s="2">
         <f t="shared" ref="F216" si="48">B216*H216*I216*J216</f>
@@ -4706,12 +4695,12 @@
         <v>1.5</v>
       </c>
       <c r="L216" s="10" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="218" spans="1:12" x14ac:dyDescent="0.2">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="218" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C218" s="2" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F218" s="2">
         <f t="shared" ref="F218" si="49">B218*H218*I218*J218</f>
@@ -4727,12 +4716,12 @@
         <v>1.5</v>
       </c>
       <c r="L218" s="10" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="220" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C220" s="2" t="s">
         <v>136</v>
-      </c>
-    </row>
-    <row r="220" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="C220" s="2" t="s">
-        <v>138</v>
       </c>
       <c r="F220" s="2">
         <f t="shared" ref="F220" si="50">B220*H220*I220*J220</f>
@@ -4748,21 +4737,21 @@
         <v>1.5</v>
       </c>
       <c r="L220" s="10" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="223" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="223" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A223" s="1">
         <v>8</v>
       </c>
       <c r="C223" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D223" s="3"/>
     </row>
-    <row r="225" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C225" s="2" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="F225" s="2">
         <f t="shared" ref="F225" si="51">B225*H225*I225*J225</f>
@@ -4778,12 +4767,12 @@
         <v>1.5</v>
       </c>
       <c r="L225" s="10" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="227" spans="1:12" x14ac:dyDescent="0.2">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="227" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C227" s="2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="F227" s="2">
         <f t="shared" ref="F227" si="52">B227*H227*I227*J227</f>
@@ -4799,12 +4788,12 @@
         <v>1.5</v>
       </c>
       <c r="L227" s="10" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="229" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C229" s="2" t="s">
         <v>142</v>
-      </c>
-    </row>
-    <row r="229" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="C229" s="2" t="s">
-        <v>144</v>
       </c>
       <c r="F229" s="2">
         <f t="shared" ref="F229" si="53">B229*H229*I229*J229</f>
@@ -4820,12 +4809,12 @@
         <v>1.5</v>
       </c>
       <c r="L229" s="10" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="231" spans="1:12" x14ac:dyDescent="0.2">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="231" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C231" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="F231" s="2">
         <f t="shared" ref="F231" si="54">B231*H231*I231*J231</f>
@@ -4841,21 +4830,21 @@
         <v>1.5</v>
       </c>
       <c r="L231" s="10" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="236" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="236" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A236" s="1">
         <v>9</v>
       </c>
       <c r="C236" s="3" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D236" s="3"/>
     </row>
-    <row r="238" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C238" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F238" s="2">
         <f t="shared" ref="F238" si="55">B238*H238*I238*J238</f>
@@ -4871,12 +4860,12 @@
         <v>1.5</v>
       </c>
       <c r="L238" s="10" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="240" spans="1:12" x14ac:dyDescent="0.2">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="240" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C240" s="2" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F240" s="2">
         <f t="shared" ref="F240" si="56">B240*H240*I240*J240</f>
@@ -4892,17 +4881,17 @@
         <v>1.5</v>
       </c>
       <c r="L240" s="10" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="241" spans="3:12" x14ac:dyDescent="0.25">
+      <c r="L241" s="10" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="243" spans="3:12" x14ac:dyDescent="0.25">
+      <c r="C243" s="2" t="s">
         <v>150</v>
-      </c>
-    </row>
-    <row r="241" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="L241" s="10" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="243" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="C243" s="2" t="s">
-        <v>152</v>
       </c>
       <c r="F243" s="2">
         <f t="shared" ref="F243" si="57">B243*H243*I243*J243</f>
@@ -4918,12 +4907,12 @@
         <v>1.5</v>
       </c>
       <c r="L243" s="10" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="245" spans="3:12" x14ac:dyDescent="0.2">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="245" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C245" s="2" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="F245" s="2">
         <f t="shared" ref="F245" si="58">B245*H245*I245*J245</f>
@@ -4939,12 +4928,12 @@
         <v>1.5</v>
       </c>
       <c r="L245" s="10" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="247" spans="3:12" x14ac:dyDescent="0.2">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="247" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C247" s="2" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="F247" s="2">
         <f t="shared" ref="F247" si="59">B247*H247*I247*J247</f>
@@ -4960,17 +4949,17 @@
         <v>1.5</v>
       </c>
       <c r="L247" s="10" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="248" spans="3:12" x14ac:dyDescent="0.2">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="248" spans="3:12" x14ac:dyDescent="0.25">
       <c r="L248" s="10" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="250" spans="3:12" x14ac:dyDescent="0.2">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="250" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C250" s="2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="F250" s="2">
         <f>B250*H250*I250*J250</f>
@@ -4986,17 +4975,17 @@
         <v>1.5</v>
       </c>
       <c r="L250" s="10" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="251" spans="3:12" x14ac:dyDescent="0.25">
+      <c r="L251" s="10" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="253" spans="3:12" x14ac:dyDescent="0.25">
+      <c r="C253" s="2" t="s">
         <v>156</v>
-      </c>
-    </row>
-    <row r="251" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="L251" s="10" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="253" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="C253" s="2" t="s">
-        <v>158</v>
       </c>
       <c r="F253" s="2">
         <f t="shared" ref="F253" si="60">B253*H253*I253*J253</f>
@@ -5012,12 +5001,12 @@
         <v>1.5</v>
       </c>
       <c r="L253" s="10" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="255" spans="3:12" x14ac:dyDescent="0.2">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="255" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C255" s="2" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="F255" s="2">
         <f t="shared" ref="F255" si="61">B255*H255*I255*J255</f>
@@ -5033,12 +5022,12 @@
         <v>1.5</v>
       </c>
       <c r="L255" s="10" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="257" spans="1:12" x14ac:dyDescent="0.2">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="257" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C257" s="2" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="F257" s="2">
         <f t="shared" ref="F257" si="62">B257*H257*I257*J257</f>
@@ -5054,17 +5043,17 @@
         <v>1.5</v>
       </c>
       <c r="L257" s="10" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="258" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C258" s="2" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="260" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C260" s="2" t="s">
         <v>163</v>
-      </c>
-    </row>
-    <row r="258" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="C258" s="2" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="260" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="C260" s="2" t="s">
-        <v>165</v>
       </c>
       <c r="F260" s="2">
         <f t="shared" ref="F260" si="63">B260*H260*I260*J260</f>
@@ -5080,17 +5069,17 @@
         <v>1.5</v>
       </c>
       <c r="L260" s="10" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="261" spans="1:12" x14ac:dyDescent="0.2">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="261" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C261" s="2" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="263" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="263" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="C263" s="12" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="D263" s="12"/>
       <c r="F263" s="2">
@@ -5107,21 +5096,21 @@
         <v>1.5</v>
       </c>
       <c r="L263" s="10" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="266" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="266" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A266" s="1">
         <v>10</v>
       </c>
       <c r="C266" s="3" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="D266" s="3"/>
     </row>
-    <row r="268" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="268" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C268" s="2" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="F268" s="2">
         <f t="shared" ref="F268" si="65">B268*H268*I268*J268</f>
@@ -5137,12 +5126,12 @@
         <v>1.2</v>
       </c>
       <c r="L268" s="10" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="270" spans="1:12" x14ac:dyDescent="0.2">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="270" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C270" s="2" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="F270" s="2">
         <f t="shared" ref="F270" si="66">B270*H270*I270*J270</f>
@@ -5158,20 +5147,20 @@
         <v>1.2</v>
       </c>
       <c r="L270" s="10" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="274" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="274" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A274" s="1">
         <v>11</v>
       </c>
       <c r="C274" s="13" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="276" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="276" spans="1:12" ht="17" x14ac:dyDescent="0.3">
       <c r="C276" s="12" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D276" s="14"/>
       <c r="E276" s="15"/>
@@ -5189,17 +5178,17 @@
         <v>1.5</v>
       </c>
       <c r="L276" s="10" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="277" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="277" spans="1:12" ht="17" x14ac:dyDescent="0.3">
       <c r="C277" s="12"/>
       <c r="D277" s="14"/>
       <c r="E277" s="15"/>
     </row>
-    <row r="278" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="278" spans="1:12" ht="17" x14ac:dyDescent="0.3">
       <c r="C278" s="12" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D278" s="14"/>
       <c r="E278" s="15"/>
@@ -5217,7 +5206,7 @@
         <v>1.5</v>
       </c>
       <c r="L278" s="10" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix pricing reference import timeout and duplicates
</commit_message>
<xml_diff>
--- a/docs/Quotation-Cost-Template-V1.1.xlsx
+++ b/docs/Quotation-Cost-Template-V1.1.xlsx
@@ -4497,27 +4497,6 @@
         <v>119</v>
       </c>
     </row>
-    <row r="196" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="C196" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="F196" s="2">
-        <f t="shared" ref="F196" si="40">B196*H196*I196*J196</f>
-        <v>0</v>
-      </c>
-      <c r="H196" s="2">
-        <v>75</v>
-      </c>
-      <c r="I196" s="2">
-        <v>1.0900000000000001</v>
-      </c>
-      <c r="J196" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="L196" s="10" t="s">
-        <v>119</v>
-      </c>
-    </row>
     <row r="198" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C198" s="2" t="s">
         <v>121</v>

</xml_diff>

<commit_message>
Add XLSX import regression coverage
</commit_message>
<xml_diff>
--- a/docs/Quotation-Cost-Template-V1.1.xlsx
+++ b/docs/Quotation-Cost-Template-V1.1.xlsx
@@ -2678,7 +2678,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2355A233-406B-9740-B1B1-24942A627A7E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2355A233-406B-9740-B1B1-24942A627A7E}">
   <dimension ref="A2:O278"/>
   <sheetFormatPr defaultColWidth="10.77734375" defaultRowHeight="15.65" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2695,11 +2695,9 @@
       <c r="A2" s="5">
         <v>1</v>
       </c>
-      <c r="B2" s="6"/>
       <c r="C2" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="7"/>
       <c r="F2" s="3" t="s">
         <v>1</v>
       </c>
@@ -2720,7 +2718,6 @@
       <c r="C4" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="8"/>
       <c r="F4" s="2">
         <f>B4*H4*I4*J4</f>
         <v>0</v>
@@ -2742,7 +2739,6 @@
       <c r="C6" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="8"/>
       <c r="F6" s="2">
         <f>B6*H6*I6*J6</f>
         <v>0</v>
@@ -2764,7 +2760,6 @@
       <c r="C8" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D8" s="8"/>
       <c r="F8" s="2">
         <f>B8*H8*I8*J8</f>
         <v>0</v>
@@ -2786,7 +2781,6 @@
       <c r="C10" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="D10" s="8"/>
       <c r="F10" s="2">
         <f>B10*H10*I10*J10</f>
         <v>0</v>
@@ -2808,7 +2802,6 @@
       <c r="C12" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="D12" s="8"/>
       <c r="F12" s="2">
         <f>B12*H12*I12*J12</f>
         <v>0</v>
@@ -2830,7 +2823,6 @@
       <c r="C14" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="D14" s="8"/>
       <c r="F14" s="2">
         <f>B14*H14*I14*J14</f>
         <v>0</v>
@@ -2855,7 +2847,6 @@
       <c r="C17" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D17" s="3"/>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C19" s="2" t="s">
@@ -3356,15 +3347,9 @@
       <c r="C81" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D81" s="3"/>
-    </row>
-    <row r="82" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
-      <c r="A82" s="1"/>
-      <c r="C82" s="3"/>
-      <c r="D82" s="3"/>
-    </row>
+    </row>
+    <row r="82" spans="1:12" ht="16.3" x14ac:dyDescent="0.25"/>
     <row r="83" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
-      <c r="A83" s="1"/>
       <c r="C83" s="2" t="s">
         <v>46</v>
       </c>
@@ -3383,7 +3368,6 @@
       </c>
     </row>
     <row r="84" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
-      <c r="A84" s="1"/>
       <c r="C84" s="2" t="s">
         <v>48</v>
       </c>
@@ -3391,11 +3375,8 @@
         <v>21</v>
       </c>
     </row>
-    <row r="85" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
-      <c r="A85" s="1"/>
-    </row>
+    <row r="85" spans="1:12" ht="16.3" x14ac:dyDescent="0.25"/>
     <row r="86" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
-      <c r="A86" s="1"/>
       <c r="C86" s="2" t="s">
         <v>46</v>
       </c>
@@ -3414,7 +3395,6 @@
       </c>
     </row>
     <row r="87" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
-      <c r="A87" s="1"/>
       <c r="C87" s="2" t="s">
         <v>31</v>
       </c>
@@ -3422,11 +3402,8 @@
         <v>49</v>
       </c>
     </row>
-    <row r="88" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
-      <c r="A88" s="1"/>
-    </row>
+    <row r="88" spans="1:12" ht="16.3" x14ac:dyDescent="0.25"/>
     <row r="89" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
-      <c r="A89" s="1"/>
       <c r="C89" s="2" t="s">
         <v>50</v>
       </c>
@@ -3445,7 +3422,6 @@
       </c>
     </row>
     <row r="90" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
-      <c r="A90" s="1"/>
       <c r="C90" s="2" t="s">
         <v>48</v>
       </c>
@@ -3453,11 +3429,8 @@
         <v>21</v>
       </c>
     </row>
-    <row r="91" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
-      <c r="A91" s="1"/>
-    </row>
+    <row r="91" spans="1:12" ht="16.3" x14ac:dyDescent="0.25"/>
     <row r="92" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
-      <c r="A92" s="1"/>
       <c r="C92" s="2" t="s">
         <v>50</v>
       </c>
@@ -3476,7 +3449,6 @@
       </c>
     </row>
     <row r="93" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
-      <c r="A93" s="1"/>
       <c r="C93" s="2" t="s">
         <v>31</v>
       </c>
@@ -3484,11 +3456,8 @@
         <v>49</v>
       </c>
     </row>
-    <row r="94" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
-      <c r="A94" s="1"/>
-    </row>
+    <row r="94" spans="1:12" ht="16.3" x14ac:dyDescent="0.25"/>
     <row r="95" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
-      <c r="A95" s="1"/>
       <c r="C95" s="2" t="s">
         <v>52</v>
       </c>
@@ -3507,7 +3476,6 @@
       </c>
     </row>
     <row r="96" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
-      <c r="A96" s="1"/>
       <c r="C96" s="2" t="s">
         <v>48</v>
       </c>
@@ -3515,11 +3483,8 @@
         <v>21</v>
       </c>
     </row>
-    <row r="97" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
-      <c r="A97" s="1"/>
-    </row>
+    <row r="97" spans="1:12" ht="16.3" x14ac:dyDescent="0.25"/>
     <row r="98" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
-      <c r="A98" s="1"/>
       <c r="C98" s="2" t="s">
         <v>52</v>
       </c>
@@ -3538,7 +3503,6 @@
       </c>
     </row>
     <row r="99" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
-      <c r="A99" s="1"/>
       <c r="C99" s="2" t="s">
         <v>31</v>
       </c>
@@ -3546,11 +3510,8 @@
         <v>49</v>
       </c>
     </row>
-    <row r="100" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
-      <c r="A100" s="1"/>
-    </row>
+    <row r="100" spans="1:12" ht="16.3" x14ac:dyDescent="0.25"/>
     <row r="101" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
-      <c r="A101" s="1"/>
       <c r="C101" s="2" t="s">
         <v>54</v>
       </c>
@@ -3571,9 +3532,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="102" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
-      <c r="A102" s="1"/>
-    </row>
+    <row r="102" spans="1:12" ht="16.3" x14ac:dyDescent="0.25"/>
     <row r="104" spans="1:12" ht="16.3" x14ac:dyDescent="0.25">
       <c r="A104" s="1">
         <v>4</v>
@@ -3581,7 +3540,6 @@
       <c r="C104" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="D104" s="3"/>
     </row>
     <row r="106" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C106" s="2" t="s">
@@ -3630,10 +3588,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="110" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="C110" s="4"/>
-      <c r="D110" s="4"/>
-    </row>
+    <row r="110" spans="1:12" x14ac:dyDescent="0.25"/>
     <row r="111" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C111" s="2" t="s">
         <v>62</v>
@@ -3813,7 +3768,6 @@
       <c r="C128" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="D128" s="3"/>
     </row>
     <row r="130" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C130" s="2" t="s">
@@ -4029,7 +3983,6 @@
       <c r="C150" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="D150" s="11"/>
       <c r="F150" s="2">
         <f t="shared" ref="F150" si="18">B150*H150*I150*J150</f>
         <v>0</v>
@@ -4054,7 +4007,6 @@
       <c r="C152" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="D152" s="3"/>
     </row>
     <row r="154" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C154" s="2" t="s">
@@ -4567,7 +4519,6 @@
       <c r="C206" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="D206" s="3"/>
     </row>
     <row r="208" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C208" s="2" t="s">
@@ -4590,9 +4541,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="209" spans="1:12" ht="16.3" x14ac:dyDescent="0.3">
-      <c r="E209"/>
-    </row>
+    <row r="209" spans="1:12" ht="16.3" x14ac:dyDescent="0.3"/>
     <row r="210" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C210" s="2" t="s">
         <v>129</v>
@@ -4726,7 +4675,6 @@
       <c r="C223" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="D223" s="3"/>
     </row>
     <row r="225" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C225" s="2" t="s">
@@ -4819,7 +4767,6 @@
       <c r="C236" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="D236" s="3"/>
     </row>
     <row r="238" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C238" s="2" t="s">
@@ -5060,7 +5007,6 @@
       <c r="C263" s="12" t="s">
         <v>165</v>
       </c>
-      <c r="D263" s="12"/>
       <c r="F263" s="2">
         <f t="shared" ref="F263" si="64">B263*H263*I263*J263</f>
         <v>0</v>
@@ -5085,7 +5031,6 @@
       <c r="C266" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="D266" s="3"/>
     </row>
     <row r="268" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C268" s="2" t="s">
@@ -5141,8 +5086,6 @@
       <c r="C276" s="12" t="s">
         <v>180</v>
       </c>
-      <c r="D276" s="14"/>
-      <c r="E276" s="15"/>
       <c r="F276" s="2">
         <f t="shared" ref="F276" si="67">B276*H276*I276*J276</f>
         <v>0</v>
@@ -5160,17 +5103,11 @@
         <v>181</v>
       </c>
     </row>
-    <row r="277" spans="1:12" ht="17" x14ac:dyDescent="0.3">
-      <c r="C277" s="12"/>
-      <c r="D277" s="14"/>
-      <c r="E277" s="15"/>
-    </row>
+    <row r="277" spans="1:12" ht="17" x14ac:dyDescent="0.3"/>
     <row r="278" spans="1:12" ht="17" x14ac:dyDescent="0.3">
       <c r="C278" s="12" t="s">
         <v>179</v>
       </c>
-      <c r="D278" s="14"/>
-      <c r="E278" s="15"/>
       <c r="F278" s="2">
         <f t="shared" ref="F278" si="68">B278*H278*I278*J278</f>
         <v>0</v>

</xml_diff>